<commit_message>
chore: sync Nova upm-release-2026.08.26-01
</commit_message>
<xml_diff>
--- a/Assets/Samples/IAPDemo/Excels/Networks/Cmds/NetworkCmds.xlsx
+++ b/Assets/Samples/IAPDemo/Excels/Networks/Cmds/NetworkCmds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SoloGames-X\nova\Assets\Samples\IAPDemo\Excels\Networks\Cmds\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63FCFE7F-44A2-436D-AC97-4AF1F021D71D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3B45BCB-102F-4EA8-BD1C-14248DD78B48}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="81">
   <si>
     <t>##comment</t>
   </si>
@@ -93,190 +93,189 @@
     <t>GameServer</t>
   </si>
   <si>
+    <t>AppsFlyerReport</t>
+  </si>
+  <si>
+    <t>Appsflyer 数据上传</t>
+  </si>
+  <si>
+    <t>/v1/user/report-appsflyer</t>
+  </si>
+  <si>
+    <t>FirebaseReport</t>
+  </si>
+  <si>
+    <t>Firebase数据上传</t>
+  </si>
+  <si>
+    <t>/v1/user/report-firebase</t>
+  </si>
+  <si>
+    <t>TGA 服务器 URL</t>
+  </si>
+  <si>
+    <t>TGAReport</t>
+  </si>
+  <si>
+    <t>TGA数据上传</t>
+  </si>
+  <si>
+    <t>GameAccountLogin</t>
+  </si>
+  <si>
+    <t>游戏登录</t>
+  </si>
+  <si>
+    <t>/v1/user/loginV1</t>
+  </si>
+  <si>
+    <t>ThirdGetProductList</t>
+  </si>
+  <si>
+    <t>三方支付-获取商品列表</t>
+  </si>
+  <si>
+    <t>ThirdVerifyIap</t>
+  </si>
+  <si>
+    <t>三方支付-校验订单</t>
+  </si>
+  <si>
+    <t>ThirdOpenURL</t>
+  </si>
+  <si>
+    <t>ThirdOpenServer</t>
+  </si>
+  <si>
+    <t>IAPServer</t>
+  </si>
+  <si>
+    <t>ThirdQueryPendingOrder</t>
+  </si>
+  <si>
+    <t>三方支付-查询支付成功未校验订单</t>
+  </si>
+  <si>
+    <t>ThirdGetPayChannelParams</t>
+  </si>
+  <si>
+    <t>三方支付-获取支付渠道参数</t>
+  </si>
+  <si>
+    <t>ThirdGetVoucherInfo</t>
+  </si>
+  <si>
+    <t>三方支付-获取代金券列表</t>
+  </si>
+  <si>
+    <t>/en/game_recharge/gift_voucher/list</t>
+  </si>
+  <si>
+    <t>ThirdGiftVoucherDeduct</t>
+  </si>
+  <si>
+    <t>三方支付-代金券核销</t>
+  </si>
+  <si>
+    <t>/en/game_recharge/gift_voucher/deduct</t>
+  </si>
+  <si>
+    <t>ThirdGiftVoucherTestGrant</t>
+  </si>
+  <si>
+    <t>三方支付-代金券测试发放</t>
+  </si>
+  <si>
+    <t>/en/game_recharge/gift_voucher/test_grant</t>
+  </si>
+  <si>
+    <t>IAPGoogleQueryPendingOrder</t>
+  </si>
+  <si>
+    <t>谷歌-查询未完成(已支付)订单列表</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/v1/mobile_pay/google/query_pending_order </t>
+  </si>
+  <si>
+    <t>IAPGoogleVerify</t>
+  </si>
+  <si>
+    <t>谷歌-普通内购验单</t>
+  </si>
+  <si>
+    <t>/v1/mobile_pay/google/verify_iap</t>
+  </si>
+  <si>
+    <t>IAPGoogleVerifySubscription</t>
+  </si>
+  <si>
+    <t>谷歌-订阅内购验单</t>
+  </si>
+  <si>
+    <t>/v1/mobile_pay/google/verify_subscribe</t>
+  </si>
+  <si>
+    <t>IAPAppleQueryPendingOrder</t>
+  </si>
+  <si>
+    <t>苹果-查询未完成(已支付)订单列表</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/v1/mobile_pay/apple/query_pending_order </t>
+  </si>
+  <si>
+    <t>IAPAppleVerify</t>
+  </si>
+  <si>
+    <t>苹果-普通内购验单</t>
+  </si>
+  <si>
+    <t>/v1/mobile_pay/apple/verify_iap</t>
+  </si>
+  <si>
+    <t>IAPAppleVerifySubscription</t>
+  </si>
+  <si>
+    <t>苹果-订阅内购验单</t>
+  </si>
+  <si>
+    <t>/v1/mobile_pay/apple/verify_subscribe</t>
+  </si>
+  <si>
+    <t>三方支付-打开支付页 URL</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>/v1/user/report-tga</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>IAPServer</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>/v1/third_pay/get_payment_customer_ids</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>/v1/third_pay/query_pending_order</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>/v1/third_pay/verify_iap</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
     <t>/v1/common/app-config</t>
-  </si>
-  <si>
-    <t>AppsFlyerReport</t>
-  </si>
-  <si>
-    <t>Appsflyer 数据上传</t>
-  </si>
-  <si>
-    <t>/v1/user/report-appsflyer</t>
-  </si>
-  <si>
-    <t>FirebaseReport</t>
-  </si>
-  <si>
-    <t>Firebase数据上传</t>
-  </si>
-  <si>
-    <t>/v1/user/report-firebase</t>
-  </si>
-  <si>
-    <t>TGA 服务器 URL</t>
-  </si>
-  <si>
-    <t>TGAReport</t>
-  </si>
-  <si>
-    <t>TGA数据上传</t>
-  </si>
-  <si>
-    <t>/v1/user/report-tga</t>
-  </si>
-  <si>
-    <t>GameAccountLogin</t>
-  </si>
-  <si>
-    <t>游戏登录</t>
-  </si>
-  <si>
-    <t>/v1/user/loginV1</t>
-  </si>
-  <si>
-    <t>ThirdGetProductList</t>
-  </si>
-  <si>
-    <t>三方支付-获取商品列表</t>
-  </si>
-  <si>
-    <t>ThirdServer</t>
-  </si>
-  <si>
-    <t>ThirdVerifyIap</t>
-  </si>
-  <si>
-    <t>三方支付-校验订单</t>
-  </si>
-  <si>
-    <t>/en/third_pay/verify_iap</t>
-  </si>
-  <si>
-    <t>ThirdOpenURL</t>
-  </si>
-  <si>
-    <t>三方支付-打开支付页 URL</t>
-  </si>
-  <si>
-    <t>ThirdOpenServer</t>
-  </si>
-  <si>
-    <t>/taylor</t>
-  </si>
-  <si>
-    <t>IAPServer</t>
-  </si>
-  <si>
-    <t>ThirdQueryPendingOrder</t>
-  </si>
-  <si>
-    <t>三方支付-查询支付成功未校验订单</t>
-  </si>
-  <si>
-    <t>/en/third_pay/query_pending_order</t>
-  </si>
-  <si>
-    <t>ThirdGetPayChannelParams</t>
-  </si>
-  <si>
-    <t>三方支付-获取支付渠道参数</t>
-  </si>
-  <si>
-    <t>/en/third_pay/get_payment_customer_ids</t>
-  </si>
-  <si>
-    <t>ThirdGetVoucherInfo</t>
-  </si>
-  <si>
-    <t>三方支付-获取代金券列表</t>
-  </si>
-  <si>
-    <t>/en/game_recharge/gift_voucher/list</t>
-  </si>
-  <si>
-    <t>ThirdGiftVoucherDeduct</t>
-  </si>
-  <si>
-    <t>三方支付-代金券核销</t>
-  </si>
-  <si>
-    <t>/en/game_recharge/gift_voucher/deduct</t>
-  </si>
-  <si>
-    <t>ThirdGiftVoucherTestGrant</t>
-  </si>
-  <si>
-    <t>三方支付-代金券测试发放</t>
-  </si>
-  <si>
-    <t>/en/game_recharge/gift_voucher/test_grant</t>
-  </si>
-  <si>
-    <t>IAPGetPayDataStatistics</t>
-  </si>
-  <si>
-    <t>官方内购-获取支付数据统计</t>
-  </si>
-  <si>
-    <t>/payment2/getPayData</t>
-  </si>
-  <si>
-    <t>IAPGoogleQueryPendingOrder</t>
-  </si>
-  <si>
-    <t>谷歌-查询未完成(已支付)订单列表</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/v1/mobile_pay/google/query_pending_order </t>
-  </si>
-  <si>
-    <t>IAPGoogleVerify</t>
-  </si>
-  <si>
-    <t>谷歌-普通内购验单</t>
-  </si>
-  <si>
-    <t>/v1/mobile_pay/google/verify_iap</t>
-  </si>
-  <si>
-    <t>IAPGoogleVerifySubscription</t>
-  </si>
-  <si>
-    <t>谷歌-订阅内购验单</t>
-  </si>
-  <si>
-    <t>/v1/mobile_pay/google/verify_subscribe</t>
-  </si>
-  <si>
-    <t>IAPAppleQueryPendingOrder</t>
-  </si>
-  <si>
-    <t>苹果-查询未完成(已支付)订单列表</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/v1/mobile_pay/apple/query_pending_order </t>
-  </si>
-  <si>
-    <t>IAPAppleVerify</t>
-  </si>
-  <si>
-    <t>苹果-普通内购验单</t>
-  </si>
-  <si>
-    <t>/v1/mobile_pay/apple/verify_iap</t>
-  </si>
-  <si>
-    <t>IAPAppleVerifySubscription</t>
-  </si>
-  <si>
-    <t>苹果-订阅内购验单</t>
-  </si>
-  <si>
-    <t>/v1/mobile_pay/apple/verify_subscribe</t>
-  </si>
-  <si>
-    <t>/en/third_pay/product_list</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>/v1/third_pay/product_list</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>/nova</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -737,7 +736,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U41"/>
+  <dimension ref="A1:U40"/>
   <sheetFormatPr defaultColWidth="13" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
@@ -869,7 +868,7 @@
         <v>15</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>16</v>
@@ -896,10 +895,10 @@
     </row>
     <row r="6" spans="1:21" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>30</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>31</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>20</v>
@@ -907,16 +906,16 @@
       <c r="E6" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="8" t="s">
-        <v>32</v>
+      <c r="F6" s="9" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>20</v>
@@ -925,15 +924,15 @@
         <v>21</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:21" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>20</v>
@@ -942,15 +941,15 @@
         <v>21</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:21" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>20</v>
@@ -959,281 +958,265 @@
         <v>21</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:21" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>38</v>
+      <c r="E11" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:21" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>44</v>
+        <v>20</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:21" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:21" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:21" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:21" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>59</v>
+        <v>34</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>61</v>
+      <c r="E17" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>64</v>
+      <c r="E18" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
-        <v>65</v>
+        <v>41</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>66</v>
+        <v>42</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>67</v>
+      <c r="E19" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>70</v>
+      <c r="E20" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C21" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="9" t="s">
         <v>72</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>73</v>
+        <v>39</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="22" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E22" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>46</v>
-      </c>
       <c r="F22" s="2" t="s">
-        <v>76</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="2" t="s">
-        <v>77</v>
+        <v>48</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>78</v>
+        <v>49</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>46</v>
+      <c r="E23" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="2" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>81</v>
+        <v>52</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>46</v>
+      <c r="E24" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1249,7 +1232,6 @@
     <row r="38" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>